<commit_message>
De 25%-reductie is het verschil tussen met en zonder zool
Rechtzetting van gisteren. Ik had de baselinemeting van visite 1 als de
referentie beschreven waartegen de reductie gerekend wordt. Dat klopt niet:
op elk meetmoment worden beide condities gemeten -- zonder de CMFO en met de
CMFO -- en de 25% is het verschil tussen die twee in dezelfde sessie.

Daarmee vervalt de vraag die ik gisteren openliet over wat er gebeurt als een
deelnemer later ander schoeisel krijgt. Er is geen oude referentie die kan
verouderen; beide condities worden dan gewoon opnieuw gemeten.

De norm luidt nu: piekdruk onder 200 kPa met de zool, of minstens 25% lager
dan dezelfde regio zonder de zool, in dezelfde sessie gemeten.

eCRF 24 moet dus twee condities vragen in plaats van drie, en beide op elk
meetmoment.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARADISE_WP1_afvinklijst.xlsx
+++ b/PARADISE_WP1_afvinklijst.xlsx
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Pedar als klinisch toestel met trublu-kalibratie; F-Scan GO alleen studieteam; acht regio's; norm &lt; 200 kPa óf ≥ 25% reductie; behaalde reductie als fidelity-maat</t>
+          <t>Pedar als klinisch toestel met trublu-kalibratie; F-Scan GO alleen studieteam; acht regio's; alles in-shoe, zónder én mét de zool gemeten; norm &lt; 200 kPa mét de zool óf ≥ 25% lager dan zonder, in dezelfde sessie; behaalde reductie als fidelity-maat</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
@@ -4277,8 +4277,8 @@
   <mergeCells count="11">
     <mergeCell ref="A65:I65"/>
     <mergeCell ref="A73:I73"/>
+    <mergeCell ref="A41:I41"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A41:I41"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A60:I60"/>
     <mergeCell ref="A1:I1"/>
@@ -4992,6 +4992,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
@@ -5008,7 +5009,7 @@
       </c>
       <c r="C28" s="23" t="inlineStr">
         <is>
-          <t>Alles in-shoe. De baseline meet zónder de CMFO, alle latere metingen mét. Tabel 4 van het manuscript had het dus goed</t>
+          <t>Alles in-shoe, twee condities: zónder en mét de CMFO. De 25%-reductie is het verschil tussen die twee, in dezelfde sessie gemeten. Tabel 4 van het manuscript had het goed</t>
         </is>
       </c>
       <c r="D28" s="23" t="inlineStr">
@@ -5074,7 +5075,7 @@
       </c>
       <c r="C30" s="23" t="inlineStr">
         <is>
-          <t>Vraagt nu drie condities; de blootsvoetse vervalt</t>
+          <t>De blootsvoetse conditie vervalt; de twee overblijvende condities worden op elk meetmoment allebei gemeten</t>
         </is>
       </c>
       <c r="D30" s="23" t="inlineStr">
@@ -5140,7 +5141,7 @@
       </c>
       <c r="C32" s="23" t="inlineStr">
         <is>
-          <t>Wordt de meting zónder zool herhaald als een deelnemer later ander schoeisel krijgt? Anders slaat de referentie op een schoen die hij niet meer draagt</t>
+          <t>Beantwoord: de meting zónder zool hoort bij elk meetmoment, dus er is geen oude referentie die kan verouderen</t>
         </is>
       </c>
       <c r="D32" s="23" t="inlineStr">
@@ -5155,12 +5156,12 @@
       </c>
       <c r="F32" s="23" t="inlineStr">
         <is>
-          <t>Te doen</t>
+          <t>Vervalt</t>
         </is>
       </c>
       <c r="G32" s="23" t="inlineStr">
         <is>
-          <t>Raakt de formule voor de 25%-reductie</t>
+          <t>Opgelost door de beslissing</t>
         </is>
       </c>
     </row>

</xml_diff>